<commit_message>
updated for PR comments
</commit_message>
<xml_diff>
--- a/rules/CORE-000091/negative/01/data/unit-test-coreid-CG0108-negative.xlsx
+++ b/rules/CORE-000091/negative/01/data/unit-test-coreid-CG0108-negative.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -53,18 +53,23 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <i/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -72,6 +77,12 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -107,14 +118,15 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,10 +469,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -484,10 +496,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>ag.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Procedure Agents</v>
       </c>
     </row>
@@ -500,7 +512,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -536,32 +548,52 @@
         <v>6</v>
       </c>
       <c r="E2" s="2" t="str">
+        <v>AGTRT</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>Tuberculin PPD-S</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="str">
+        <v>ag.xpt</v>
+      </c>
+      <c r="C3" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="4">
+        <v>6</v>
+      </c>
+      <c r="E3" s="4" t="str">
         <v>AGTRTV</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2">
+    <row r="4">
+      <c r="A4" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>ag.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C4" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D4" s="4">
         <v>6</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E4" s="4" t="str">
         <v>AGVAMTU</v>
       </c>
-      <c r="F3" s="2" t="str">
+      <c r="F4" s="4" t="str">
         <v>mL</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -609,270 +641,270 @@
       </c>
     </row>
     <row r="2" xml:space="preserve">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="4" t="str">
+      <c r="D2" s="6" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="4" t="str">
+      <c r="E2" s="6" t="str">
         <v>Reported Agent Name</v>
       </c>
-      <c r="F2" s="4" t="str">
+      <c r="F2" s="6" t="str">
         <v>AG Pre-Specified</v>
       </c>
-      <c r="G2" s="4" t="str">
+      <c r="G2" s="6" t="str">
         <v>AG Occurrence</v>
       </c>
-      <c r="H2" s="4" t="str">
+      <c r="H2" s="6" t="str">
         <v>Dose per Administration</v>
       </c>
-      <c r="I2" s="4" t="str">
+      <c r="I2" s="6" t="str">
         <v>Dose Units</v>
       </c>
-      <c r="J2" s="4" t="str">
+      <c r="J2" s="6" t="str">
         <v>Treatment Vehicle</v>
       </c>
-      <c r="K2" s="4" t="str" xml:space="preserve">
+      <c r="K2" s="6" t="str" xml:space="preserve">
         <v xml:space="preserve">Treatment Vehicle
 Amount</v>
       </c>
-      <c r="L2" s="4" t="str" xml:space="preserve">
+      <c r="L2" s="6" t="str" xml:space="preserve">
         <v xml:space="preserve">Treatment Vehicle
 Amount Units</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="str">
+      <c r="A3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="4" t="str">
+      <c r="B3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="4" t="str">
+      <c r="C3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="4" t="str">
+      <c r="D3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="4" t="str">
+      <c r="E3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="F3" s="4" t="str">
+      <c r="F3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="G3" s="4" t="str">
+      <c r="G3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="H3" s="4" t="str">
+      <c r="H3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="I3" s="4" t="str">
+      <c r="I3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="J3" s="4" t="str">
+      <c r="J3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="K3" s="4" t="str">
+      <c r="K3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="L3" s="4" t="str">
+      <c r="L3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4">
+      <c r="A4" s="6">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6">
         <v>8</v>
       </c>
-      <c r="E4" s="4">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4">
-        <v>50</v>
-      </c>
-      <c r="H4" s="4">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4">
-        <v>50</v>
-      </c>
-      <c r="K4" s="4">
-        <v>50</v>
-      </c>
-      <c r="L4" s="4">
+      <c r="E4" s="6">
+        <v>50</v>
+      </c>
+      <c r="F4" s="6">
+        <v>50</v>
+      </c>
+      <c r="G4" s="6">
+        <v>50</v>
+      </c>
+      <c r="H4" s="6">
+        <v>50</v>
+      </c>
+      <c r="I4" s="6">
+        <v>50</v>
+      </c>
+      <c r="J4" s="6">
+        <v>50</v>
+      </c>
+      <c r="K4" s="6">
+        <v>50</v>
+      </c>
+      <c r="L4" s="6">
         <v>50</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="str">
+      <c r="A5" s="4" t="str">
         <v>XYZ</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="4" t="str">
         <v>AG</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="4" t="str">
         <v>XYZ-001-001</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="4" t="str">
         <v>Tuberculin PPD-S</v>
       </c>
-      <c r="F5" s="2" t="str">
+      <c r="F5" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G5" s="2" t="str">
+      <c r="G5" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="4">
         <v>5</v>
       </c>
-      <c r="I5" s="2" t="str">
+      <c r="I5" s="4" t="str">
         <v>tuberculin unit</v>
       </c>
-      <c r="J5" s="2" t="str">
+      <c r="J5" s="4" t="str">
         <v>SALINE</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="4">
         <v>0.1</v>
       </c>
-      <c r="L5" s="2" t="str">
+      <c r="L5" s="4" t="str">
         <v>mL</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="str">
+      <c r="A6" s="4" t="str">
         <v>XYZ</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="4" t="str">
         <v>AG</v>
       </c>
-      <c r="C6" s="2" t="str">
+      <c r="C6" s="4" t="str">
         <v>XYZ-001-002</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="4">
         <v>1</v>
       </c>
-      <c r="E6" s="2" t="str">
+      <c r="E6" s="7" t="str">
         <v>Tuberculin PPD-S</v>
       </c>
-      <c r="F6" s="2" t="str">
+      <c r="F6" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G6" s="2" t="str">
+      <c r="G6" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="4">
         <v>5</v>
       </c>
-      <c r="I6" s="2" t="str">
+      <c r="I6" s="4" t="str">
         <v>tuberculin unit</v>
       </c>
-      <c r="J6" s="6" t="str">
+      <c r="J6" s="7" t="str">
         <v/>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="4">
         <v>0.1</v>
       </c>
-      <c r="L6" s="6" t="str">
+      <c r="L6" s="7" t="str">
         <v>mL</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="str">
+      <c r="A7" s="4" t="str">
         <v>XYZ</v>
       </c>
-      <c r="B7" s="2" t="str">
+      <c r="B7" s="4" t="str">
         <v>AG</v>
       </c>
-      <c r="C7" s="2" t="str">
+      <c r="C7" s="4" t="str">
         <v>XYZ-001-002</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="4">
         <v>1</v>
       </c>
-      <c r="E7" s="2" t="str">
+      <c r="E7" s="4" t="str">
         <v>Tuberculin PPD-S</v>
       </c>
-      <c r="F7" s="2" t="str">
+      <c r="F7" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G7" s="2" t="str">
+      <c r="G7" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="4">
         <v>5</v>
       </c>
-      <c r="I7" s="2" t="str">
+      <c r="I7" s="4" t="str">
         <v>tuberculin unit</v>
       </c>
-      <c r="J7" s="5" t="str">
+      <c r="J7" s="4" t="str">
         <v>SALINE</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="4">
         <v>0.1</v>
       </c>
-      <c r="L7" s="5" t="str">
+      <c r="L7" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="str">
+      <c r="A8" s="4" t="str">
         <v>XYZ</v>
       </c>
-      <c r="B8" s="2" t="str">
+      <c r="B8" s="4" t="str">
         <v>AG</v>
       </c>
-      <c r="C8" s="2" t="str">
+      <c r="C8" s="4" t="str">
         <v>XYZ-001-002</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="4">
         <v>1</v>
       </c>
-      <c r="E8" s="2" t="str">
+      <c r="E8" s="4" t="str">
         <v>Tuberculin PPD-S</v>
       </c>
-      <c r="F8" s="2" t="str">
+      <c r="F8" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G8" s="2" t="str">
+      <c r="G8" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="4">
         <v>5</v>
       </c>
-      <c r="I8" s="2" t="str">
+      <c r="I8" s="4" t="str">
         <v>tuberculin unit</v>
       </c>
-      <c r="J8" s="5" t="str">
+      <c r="J8" s="4" t="str">
         <v/>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="4">
         <v>0.1</v>
       </c>
-      <c r="L8" s="5" t="str">
+      <c r="L8" s="4" t="str">
         <v/>
       </c>
     </row>

</xml_diff>